<commit_message>
Atualizar restos.xlsx - 16/09/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -60326,13 +60326,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23EA01ED-053D-4A51-93E4-68E532926117}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EADAF7AD-82E8-4364-B519-FEEA3E22D1E6}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3AC91BDD-72DE-47AE-9584-6C048D3119FE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C990C6D6-9D56-47CA-B805-F4D359F8C9EE}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E733CADE-6373-4FB5-B0F7-9779E5321D27}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A7AAAED-DD66-489A-B89C-29F89232DB84}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 21/09/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -60683,13 +60683,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A698672E-1CB2-4356-9B67-13E7DF78E028}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E748F3B5-3087-4978-8AE1-9776FB7B9F66}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{641FF255-129A-44D7-BFE6-C24AA0CB1497}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC99A43A-A5AA-46BC-9ED7-5DE2BB25D1FC}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F13CD093-32AB-4769-9172-DCDB99602E1B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DC1E0C-A011-4808-AF8C-96D75C943508}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 25/09/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -60683,13 +60683,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E748F3B5-3087-4978-8AE1-9776FB7B9F66}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4ADCE4B-0DC9-4D46-8A22-45ADAA194FDA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC99A43A-A5AA-46BC-9ED7-5DE2BB25D1FC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E15E26E-D1A0-4B25-B4DC-B7CFC71348FD}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5DC1E0C-A011-4808-AF8C-96D75C943508}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A196DEBF-008E-4258-A13F-0F6EE9609A88}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 28/09/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -60683,13 +60683,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C4ADCE4B-0DC9-4D46-8A22-45ADAA194FDA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C0F3F13-E496-475D-AC73-C928DD2FDC37}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E15E26E-D1A0-4B25-B4DC-B7CFC71348FD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF3EE39D-D1BA-47E2-8AD2-1DE61C79228C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A196DEBF-008E-4258-A13F-0F6EE9609A88}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77FF291D-97FC-44FE-846E-E1775F14024D}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 05/10/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -61505,13 +61505,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A86DF94-1E9D-4DC9-BFD3-0F92A7901C0A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA80FD38-B84B-49F0-86DA-0CDE72C392D9}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A26A449-EEF4-49BF-9F4D-B481C72727E9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98B119D4-7557-4F68-9DEC-E316D65F418E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA82EEC2-642F-4FE8-A2D5-4B681A9065D5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{145E4A7E-DD6D-49F3-BE61-737459A85A9A}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 06/10/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -61505,13 +61505,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA80FD38-B84B-49F0-86DA-0CDE72C392D9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75442760-8117-495E-804B-303B44F8623A}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98B119D4-7557-4F68-9DEC-E316D65F418E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{832A9333-2932-4559-B76F-0528314DC7E4}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{145E4A7E-DD6D-49F3-BE61-737459A85A9A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{458E8170-36D8-4FCE-8677-8753188A5786}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 08/10/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -61505,13 +61505,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75442760-8117-495E-804B-303B44F8623A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F09DBD24-4E3F-4BAC-9533-BC6CBF49BC45}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{832A9333-2932-4559-B76F-0528314DC7E4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37969524-FACC-4388-8083-0D04C67BE82A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{458E8170-36D8-4FCE-8677-8753188A5786}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52D3F2FC-E237-4B70-843B-B6900CD12BCE}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 09/10/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -61505,13 +61505,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F09DBD24-4E3F-4BAC-9533-BC6CBF49BC45}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{527FA720-A938-4D16-83B1-40636B202FCE}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37969524-FACC-4388-8083-0D04C67BE82A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8450B8DB-13E1-415F-ADA3-85A0F5094761}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52D3F2FC-E237-4B70-843B-B6900CD12BCE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5609E2A-0A58-44CE-8D1D-31A6CE8AA2BF}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 15/10/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -61505,13 +61505,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{527FA720-A938-4D16-83B1-40636B202FCE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD641857-6550-423D-B06B-549BCAB19E75}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8450B8DB-13E1-415F-ADA3-85A0F5094761}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{316A4DDC-DA4B-45AD-8A2F-5F7E162B8DAB}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5609E2A-0A58-44CE-8D1D-31A6CE8AA2BF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91889D9A-4114-46E8-8F1C-5774C12760D2}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 16/10/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -541,7 +541,7 @@
     <t>LOCACAO DE SERVICOS DE CONSERVACAO E LIMPEZA REALIZADOS PELA MGS</t>
   </si>
   <si>
-    <t>Pendente de transmissão aos bancos</t>
+    <t>Transmitida ao banco - Pendente de Confirmação</t>
   </si>
   <si>
     <t>LOCACAO DE SERVICOS DE APOIO ADMINISTRATIVO REALIZADOS PELA MGS</t>
@@ -1454,7 +1454,7 @@
     <col min="2" max="19" width="10.7163133333333" customWidth="1"/>
     <col min="20" max="20" width="20.9645" customWidth="1"/>
     <col min="21" max="22" width="10.7163133333333" customWidth="1"/>
-    <col min="23" max="23" width="34.2738333333333" customWidth="1"/>
+    <col min="23" max="23" width="42.2594333333333" customWidth="1"/>
     <col min="24" max="32" width="10.7163133333333" customWidth="1"/>
     <col min="33" max="33" width="22.4855666666667" customWidth="1"/>
     <col min="34" max="34" width="18.4927666666667" customWidth="1"/>
@@ -17914,7 +17914,7 @@
         <v>47</v>
       </c>
       <c r="AC146" s="4" t="s">
-        <v>47</v>
+        <v>153</v>
       </c>
       <c r="AD146" s="3">
         <v>10</v>
@@ -18033,7 +18033,7 @@
         <v>47</v>
       </c>
       <c r="AC147" s="4" t="s">
-        <v>47</v>
+        <v>153</v>
       </c>
       <c r="AD147" s="3">
         <v>10</v>
@@ -45504,7 +45504,7 @@
         <v>47</v>
       </c>
       <c r="AC384" s="4" t="s">
-        <v>47</v>
+        <v>153</v>
       </c>
       <c r="AD384" s="3">
         <v>10</v>
@@ -57183,7 +57183,7 @@
         <v>47</v>
       </c>
       <c r="AC485" s="4" t="s">
-        <v>47</v>
+        <v>153</v>
       </c>
       <c r="AD485" s="3">
         <v>10</v>
@@ -57536,7 +57536,7 @@
         <v>47</v>
       </c>
       <c r="AC488" s="4" t="s">
-        <v>47</v>
+        <v>153</v>
       </c>
       <c r="AD488" s="3">
         <v>10</v>
@@ -62450,13 +62450,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E9B660B-D1C3-48FB-ABB7-1A345DF9A033}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7D980F0-49E0-484D-BC39-FEED4E302613}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{613CDDF1-417D-4870-8D2A-CD11B329E987}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5115218-B91C-40C4-ADB0-932021E03605}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{25A07257-D7A6-4180-957A-6C8D6A1A2425}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4D43860-CBC4-42A4-9D22-EF79DAB11C93}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 22/10/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -63597,13 +63597,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D10EEFD-7EB6-49AE-94B1-46BD17CAF209}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46AEF257-1200-4E69-A4BE-45D862DED09C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{673C6D4D-9773-4D86-8EE0-DD2C5B2AA078}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F1BEE0C-7E05-4121-BC54-AE9434A31050}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35B5FFFB-200D-4769-8B38-5089D25A5BCC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2812DC98-4AD1-47E7-AF7A-AEA289269F81}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 26/10/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -16468,7 +16468,7 @@
         <v>0</v>
       </c>
       <c r="T134" s="5">
-        <v>-8261.32</v>
+        <v>-9124.46</v>
       </c>
       <c r="U134" s="3">
         <v>0</v>
@@ -16503,7 +16503,7 @@
         <v>1.480004e6</v>
       </c>
       <c r="AG134" s="5">
-        <v>8261.32</v>
+        <v>9124.46</v>
       </c>
       <c r="AH134" s="5">
         <v>0</v>
@@ -63597,13 +63597,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46AEF257-1200-4E69-A4BE-45D862DED09C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EC1955F1-D6FC-4442-B486-685DB3B5EEA0}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F1BEE0C-7E05-4121-BC54-AE9434A31050}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21B73D30-43A5-4BFC-9147-90E10DCE6DC4}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2812DC98-4AD1-47E7-AF7A-AEA289269F81}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{023155DB-4AD2-45AD-AF9D-067C3AC53BB2}"/>
 </file>
</xml_diff>